<commit_message>
save 08 04 2026
</commit_message>
<xml_diff>
--- a/4 четверть_9_JavaScript_Vue.xlsx
+++ b/4 четверть_9_JavaScript_Vue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45559D31-AAFB-4191-8C89-562D186D0B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0D4ED4-F60B-426D-BFC4-11E4C350C1F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2790" yWindow="-17325" windowWidth="27330" windowHeight="12000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Название 1-3" sheetId="12" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="515">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -8017,17 +8017,611 @@
 &lt;/script&gt;</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    &lt;div class="gr-bd_content_receiveraddmenu" &gt;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">        &lt;transition name="</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>slide-fade</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+            </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;ReceiverAddMenu</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+                </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>v-if="mods.modAddReceiver"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+                :mailReceiversInGrp="mailReceiversInGrp"
+                :groupSelected="groupSelected"
+                @updateAllMailReceiversByGroupId="getAllMailReceiversByGroupId()"
+                @updateGroupsOfMlRcvs="updateGroupsOfMlRcvs()"
+                @exitReceiverAddMenu="Object.set(mods, 'modAddReceiver', false);"
+            </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&gt;&lt;/ReceiverAddMenu&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">        &lt;/transition&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    &lt;/div&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Когда нужно!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Когда используется v-if, однако требуется анимация. Если использовать нативный подход, анимация не сработает. В связи с этим необходимо использовать встроенный компонент </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>transition</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Пояснение! </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>transition</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> должен выступать оберткой компонента, который необходимо анимировать.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>v-if</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> указывается на компоненте-потомке </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>transition</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        &amp;_receiveraddmenu {
+            position: absolute;
+            top: 0px;
+            left: 0px;
+            width: 100%;
+            background-color: transparent;
+            z-index: 1;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">            &amp; .slide-fade-enter-active,
+            &amp; .slide-fade-leave-active {
+              transition: transform 0.7s ease;
+              will-change: transform; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/* Оптимизация для браузера */</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+            }
+            &amp; .slide-fade-enter,
+            &amp; .slide-fade-leave-to {
+              transform: translateX(100%);</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> //появление справа-налево</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+              transform: translateX(-100%); </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>//появление слева-направо</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+            }
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+            &amp; .anchor {
+                position: relative;
+                z-index: 2;
+                &amp; .component-exit {
+                    position: absolute;
+                    left: 0px;
+                    top: 5px;
+                    width: 50px;
+                    height: 35px;
+                    background-color: #182649;
+                    border-radius: 20px;
+                    color: white;
+                    display: flex;
+                    align-items: center;
+                    padding-left: 7px;
+                    z-index: -1;
+                    cursor: pointer;
+                }
+                &amp; .ra-menu_container {
+                    width: calc(100% - 26px);
+                    height: 475px;
+                    background-color: white;
+                    -webkit-box-shadow: -35px 0px 40px -13px rgba(34, 60, 80, 0.27);
+                    -moz-box-shadow: -35px 0px 40px -13px rgba(34, 60, 80, 0.27);
+                    box-shadow: 0 5px 30px 0 rgba(0,0,0,0.2);
+                    margin: 30px 10px 20px 25px;
+                    padding: 10px 20px;
+                    z-index: 2;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Анимация</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Как должна работать анимация при первом вызове (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.slide-fade-enter-active</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) анимации и при втором вызове (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.slide-fade-leave-active</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&amp; .slide-fade-enter-active,
+&amp; .slide-fade-leave-active {
+ transition: transform 0.7s ease;
+ will-change: transform; 
+}
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Где должен располагаться элемент перед(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.slide-fade-enter</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)/после(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.slide-fade-leave-to</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) анимации</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&amp; .slide-fade-enter,
+&amp; .slide-fade-leave-to {
+ transform: translateX(100%); //появление справа-налево
+ transform: translateX(-100%); //появление слева-направо
+}</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="40">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -8449,11 +9043,11 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -8464,20 +9058,20 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -8489,7 +9083,7 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -8498,80 +9092,83 @@
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="18" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="12" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="12" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="14" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="17" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="34" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="12" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="12" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="14" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="33" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -8580,28 +9177,43 @@
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -8610,68 +9222,53 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="39" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="9" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="3" applyFill="1"/>
+    <xf numFmtId="49" fontId="2" fillId="10" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="10" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="11" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="13" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="3" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="10" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="10" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="11" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="13" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Гиперссылка" xfId="2" builtinId="8"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 2" xfId="1" xr:uid="{141A142D-D8A7-43F9-B8D2-54AA311FA1CB}"/>
     <cellStyle name="Обычный 2 2" xfId="3" xr:uid="{C739D4B1-2A16-47B8-8914-B47AE649C078}"/>
   </cellStyles>
@@ -9746,7 +10343,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V283"/>
+  <dimension ref="A2:V285"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -12051,13 +12648,13 @@
       </c>
       <c r="C272" s="1"/>
     </row>
-    <row r="273" spans="1:3" ht="28.8">
+    <row r="273" spans="1:4" ht="28.8">
       <c r="A273" s="2"/>
       <c r="C273" s="44" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="274" spans="1:3" ht="57.6">
+    <row r="274" spans="1:4" ht="57.6">
       <c r="A274" s="44" t="s">
         <v>439</v>
       </c>
@@ -12065,74 +12662,94 @@
         <v>440</v>
       </c>
     </row>
-    <row r="275" spans="1:3">
-      <c r="A275" s="12" t="s">
+    <row r="275" spans="1:4">
+      <c r="A275" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="C275" s="44"/>
+    </row>
+    <row r="276" spans="1:4" ht="409.6">
+      <c r="A276" s="74" t="s">
+        <v>512</v>
+      </c>
+      <c r="B276" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="C276" s="74" t="s">
+        <v>513</v>
+      </c>
+      <c r="D276" s="74" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="277" spans="1:4">
+      <c r="A277" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="B275" s="2" t="s">
+      <c r="B277" s="41" t="s">
         <v>451</v>
       </c>
-      <c r="C275" s="44"/>
-    </row>
-    <row r="276" spans="1:3" ht="30">
-      <c r="A276" s="2" t="s">
+      <c r="C277" s="44"/>
+    </row>
+    <row r="278" spans="1:4" ht="30">
+      <c r="A278" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="B276" s="2" t="s">
+      <c r="B278" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="C276" s="45" t="s">
+      <c r="C278" s="45" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="277" spans="1:3" ht="60">
-      <c r="A277" s="2" t="s">
+    <row r="279" spans="1:4" ht="60">
+      <c r="A279" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="C277" s="45" t="s">
+      <c r="C279" s="45" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="278" spans="1:3" ht="45">
-      <c r="A278" s="2" t="s">
+    <row r="280" spans="1:4" ht="45">
+      <c r="A280" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="C278" s="45" t="s">
+      <c r="C280" s="45" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="279" spans="1:3" ht="28.8">
-      <c r="A279" s="2" t="s">
+    <row r="281" spans="1:4" ht="28.8">
+      <c r="A281" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="B279" s="2" t="s">
+      <c r="B281" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="C279" s="44"/>
-    </row>
-    <row r="280" spans="1:3">
-      <c r="A280" s="2"/>
-      <c r="C280" s="44"/>
-    </row>
-    <row r="281" spans="1:3">
-      <c r="A281" s="2"/>
       <c r="C281" s="44"/>
     </row>
-    <row r="282" spans="1:3" ht="302.39999999999998">
-      <c r="B282" s="2" t="s">
+    <row r="282" spans="1:4">
+      <c r="A282" s="2"/>
+      <c r="C282" s="44"/>
+    </row>
+    <row r="283" spans="1:4">
+      <c r="A283" s="2"/>
+      <c r="C283" s="44"/>
+    </row>
+    <row r="284" spans="1:4" ht="302.39999999999998">
+      <c r="B284" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="C282" s="46" t="s">
+      <c r="C284" s="46" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="283" spans="1:3" ht="216">
-      <c r="C283" s="46" t="s">
+    <row r="285" spans="1:4" ht="216">
+      <c r="C285" s="46" t="s">
         <v>441</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -12147,82 +12764,82 @@
   <dimension ref="A1:V14"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="36" style="66" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" style="67" customWidth="1"/>
-    <col min="3" max="3" width="100.44140625" style="67" customWidth="1"/>
-    <col min="4" max="4" width="56.44140625" style="66" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" style="65" customWidth="1"/>
-    <col min="6" max="6" width="43.21875" style="66" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.109375" style="67" customWidth="1"/>
-    <col min="8" max="8" width="67.88671875" style="66" customWidth="1"/>
-    <col min="9" max="9" width="64.33203125" style="66" customWidth="1"/>
-    <col min="10" max="10" width="7.77734375" style="65" customWidth="1"/>
-    <col min="11" max="11" width="39.21875" style="66" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.88671875" style="66" customWidth="1"/>
-    <col min="13" max="13" width="72.6640625" style="66" customWidth="1"/>
-    <col min="14" max="14" width="43.88671875" style="66" customWidth="1"/>
-    <col min="15" max="15" width="7.77734375" style="65" customWidth="1"/>
-    <col min="16" max="16" width="56.77734375" style="67" customWidth="1"/>
-    <col min="17" max="17" width="46.77734375" style="67" customWidth="1"/>
-    <col min="18" max="18" width="62.88671875" style="67" customWidth="1"/>
-    <col min="19" max="19" width="49.21875" style="66" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" style="68"/>
-    <col min="21" max="21" width="67.77734375" style="67" customWidth="1"/>
-    <col min="22" max="22" width="68.33203125" style="66" customWidth="1"/>
-    <col min="23" max="24" width="59.33203125" style="66" customWidth="1"/>
-    <col min="25" max="25" width="59.6640625" style="66" customWidth="1"/>
-    <col min="26" max="26" width="99.44140625" style="66" customWidth="1"/>
-    <col min="27" max="27" width="41.21875" style="66" customWidth="1"/>
-    <col min="28" max="16384" width="8.77734375" style="66"/>
+    <col min="1" max="1" width="36" style="63" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="64" customWidth="1"/>
+    <col min="3" max="3" width="100.44140625" style="64" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="63" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="62" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="63" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="64" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="63" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="63" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="62" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="63" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="63" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="63" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="63" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="62" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="64" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="64" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="64" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="63" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="65"/>
+    <col min="21" max="21" width="67.77734375" style="64" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="63" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="63" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="63" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="63" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="63" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="63"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="64"/>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
+      <c r="A1" s="71"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="69"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="70"/>
-      <c r="S2" s="70"/>
-      <c r="U2" s="70"/>
+      <c r="A2" s="66"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="K2" s="66"/>
+      <c r="L2" s="66"/>
+      <c r="M2" s="66"/>
+      <c r="N2" s="66"/>
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67"/>
+      <c r="R2" s="67"/>
+      <c r="S2" s="67"/>
+      <c r="U2" s="67"/>
     </row>
     <row r="3" spans="1:22">
-      <c r="C3" s="71" t="s">
+      <c r="C3" s="68" t="s">
         <v>463</v>
       </c>
-      <c r="P3" s="66"/>
-      <c r="U3" s="66"/>
-      <c r="V3" s="67"/>
+      <c r="P3" s="63"/>
+      <c r="U3" s="63"/>
+      <c r="V3" s="64"/>
     </row>
     <row r="4" spans="1:22">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="69" t="s">
         <v>492</v>
       </c>
-      <c r="P4" s="66"/>
-      <c r="U4" s="66"/>
-      <c r="V4" s="67"/>
+      <c r="P4" s="63"/>
+      <c r="U4" s="63"/>
+      <c r="V4" s="64"/>
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="1"/>
       <c r="B5" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="C5" s="73" t="s">
+      <c r="C5" s="70" t="s">
         <v>494</v>
       </c>
       <c r="D5" s="2"/>
@@ -12232,7 +12849,7 @@
       <c r="B6" s="2" t="s">
         <v>495</v>
       </c>
-      <c r="C6" s="73" t="s">
+      <c r="C6" s="70" t="s">
         <v>496</v>
       </c>
       <c r="D6" s="2"/>
@@ -12242,7 +12859,7 @@
       <c r="B7" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="C7" s="73" t="s">
+      <c r="C7" s="70" t="s">
         <v>498</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -12250,11 +12867,11 @@
       </c>
     </row>
     <row r="8" spans="1:22">
-      <c r="A8" s="72" t="s">
+      <c r="A8" s="69" t="s">
         <v>499</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="73"/>
+      <c r="C8" s="70"/>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:22">
@@ -12264,7 +12881,7 @@
       <c r="B9" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="C9" s="73" t="s">
+      <c r="C9" s="70" t="s">
         <v>502</v>
       </c>
       <c r="D9" s="2"/>
@@ -12276,7 +12893,7 @@
       <c r="B10" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="C10" s="73" t="s">
+      <c r="C10" s="70" t="s">
         <v>504</v>
       </c>
       <c r="D10" s="2"/>
@@ -12288,7 +12905,7 @@
       <c r="B11" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="C11" s="73" t="s">
+      <c r="C11" s="70" t="s">
         <v>506</v>
       </c>
       <c r="D11" s="2"/>
@@ -12300,7 +12917,7 @@
       <c r="B12" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="C12" s="73" t="s">
+      <c r="C12" s="70" t="s">
         <v>507</v>
       </c>
       <c r="D12" s="1"/>
@@ -12312,7 +12929,7 @@
       <c r="B13" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="C13" s="73" t="s">
+      <c r="C13" s="70" t="s">
         <v>509</v>
       </c>
       <c r="D13" s="1"/>
@@ -12324,7 +12941,7 @@
       <c r="B14" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="C14" s="67" t="s">
+      <c r="C14" s="64" t="s">
         <v>510</v>
       </c>
     </row>
@@ -12375,10 +12992,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="62"/>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
+      <c r="A1" s="72"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" s="22"/>
@@ -12534,10 +13151,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="62"/>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
+      <c r="A1" s="72"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" s="22"/>
@@ -12617,10 +13234,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="62"/>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
+      <c r="A1" s="72"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" s="22"/>
@@ -12760,10 +13377,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="62"/>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
+      <c r="A1" s="72"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" s="22"/>
@@ -12908,12 +13525,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="73" t="s">
         <v>184</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" s="22"/>
@@ -13025,10 +13642,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="62"/>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
+      <c r="A1" s="72"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" s="22"/>

</xml_diff>